<commit_message>
Update hero UI and Hindu deity prompt styling.
Fix View Showcase to scroll to #showcase, update badge copy to 3D print anywhere with cube icon, and append barefoot/no-footwear instructions to Lord/Goddess rows in character prompts spreadsheet.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/character-prompts-v3.xlsx
+++ b/public/character-prompts-v3.xlsx
@@ -1375,7 +1375,7 @@
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>Create a 3D toy model of a cartoon-style divine prince with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. He has a serene noble expression, a jeweled crown, and blue skin (traditional depiction). He wears a full golden dhoti with an ornate waistband, a royal chest piece with jewels, wrist bangles, and sandals. He holds a large decorative bow with an arrow ready, or the bow resting at his side. Decorated with lotus and gem motifs. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing.</t>
+          <t>Create a 3D toy model of a cartoon-style divine prince with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. He has a serene noble expression, a jeweled crown, and blue skin (traditional depiction). He wears a full golden dhoti with an ornate waistband, a royal chest piece with jewels, wrist bangles, and sandals. He holds a large decorative bow with an arrow ready, or the bow resting at his side. Decorated with lotus and gem motifs. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing. Character should be barefoot with no footwear (no shoes, slippers, or sandals).</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Create a 3D toy model of a cartoon-style divine cowherd boy with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. He has a playful joyful expression, a peacock feather in his crown, and blue skin (traditional depiction). He wears a full yellow dhoti, a golden chest ornament, flower garlands, wrist bangles, and anklets. He holds a small golden flute to his lips. Decorated with lotus motifs. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing.</t>
+          <t>Create a 3D toy model of a cartoon-style divine cowherd boy with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. He has a playful joyful expression, a peacock feather in his crown, and blue skin (traditional depiction). He wears a full yellow dhoti, a golden chest ornament, flower garlands, wrist bangles, and anklets. He holds a small golden flute to his lips. Decorated with lotus motifs. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing. Character should be barefoot with no footwear (no shoes, slippers, or sandals).</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>Create a 3D toy model of a cartoon-style monkey-warrior deity with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. He has a noble determined expression, a monkey face with an orange-red tinted body. He wears a full dhoti with a golden waistband, a sacred thread across his chest, wrist bangles, anklets, and a spiked mace (gada) held upright. A long curled tail behind him. Decorated with lotus and flame motifs. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing.</t>
+          <t>Create a 3D toy model of a cartoon-style monkey-warrior deity with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. He has a noble determined expression, a monkey face with an orange-red tinted body. He wears a full dhoti with a golden waistband, a sacred thread across his chest, wrist bangles, anklets, and a spiked mace (gada) held upright. A long curled tail behind him. Decorated with lotus and flame motifs. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing. Character should be barefoot with no footwear (no shoes, slippers, or sandals).</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="D43" s="17" t="inlineStr">
         <is>
-          <t>Create a 3D toy model of a cartoon-style divine warrior goddess with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. She has a serene powerful expression, long flowing dark hair, a jeweled crown, and a warm golden complexion. She has multiple arms (6 or 8), each holding a divine weapon — a trident, a lotus flower, a conch, a bow, a sword, and a chakra. She wears a full-length ornate red saree with a golden border, a jeweled chest piece, wrist bangles, anklets, and sandals. She stands on a stylized lion pedestal. Decorated with lotus motifs and a glowing halo. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing.</t>
+          <t>Create a 3D toy model of a cartoon-style divine warrior goddess with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. She has a serene powerful expression, long flowing dark hair, a jeweled crown, and a warm golden complexion. She has multiple arms (6 or 8), each holding a divine weapon — a trident, a lotus flower, a conch, a bow, a sword, and a chakra. She wears a full-length ornate red saree with a golden border, a jeweled chest piece, wrist bangles, anklets, and sandals. She stands on a stylized lion pedestal. Decorated with lotus motifs and a glowing halo. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing. Character should be barefoot with no footwear (no shoes, slippers, or sandals).</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>Create a 3D toy model of a cartoon-style divine knowledge goddess with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. She has a serene graceful expression, long flowing dark hair adorned with white flowers, a jeweled crown, and a fair golden complexion. She has four arms — holding a veena (string instrument) in two hands, a book in one, and a rosary in the other. She wears a full-length pristine white saree with a golden border, pearl jewelry, wrist bangles, and sandals. She sits on a white lotus. Decorated with swan motifs, lotus flowers, and a soft glowing halo. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing.</t>
+          <t>Create a 3D toy model of a cartoon-style divine knowledge goddess with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. She has a serene graceful expression, long flowing dark hair adorned with white flowers, a jeweled crown, and a fair golden complexion. She has four arms — holding a veena (string instrument) in two hands, a book in one, and a rosary in the other. She wears a full-length pristine white saree with a golden border, pearl jewelry, wrist bangles, and sandals. She sits on a white lotus. Decorated with swan motifs, lotus flowers, and a soft glowing halo. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing. Character should be barefoot with no footwear (no shoes, slippers, or sandals).</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="D45" s="17" t="inlineStr">
         <is>
-          <t>Create a 3D toy model of a cartoon-style divine prosperity goddess with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. She has a blissful gentle expression, long flowing dark hair, a jeweled crown, and a radiant golden complexion. She has four arms — two hands showering golden coins, one holding a lotus flower, and one in a blessing gesture. She wears a full-length rich red-and-gold saree with an ornate border, a jeweled chest piece, wrist bangles, gold anklets, and sandals. She stands on a large pink lotus. Decorated with lotus motifs, gold coins, and a warm glowing halo. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing.</t>
+          <t>Create a 3D toy model of a cartoon-style divine prosperity goddess with child-friendly, rounded toy-like proportions with a small compact body, a slightly larger head, and age-appropriate modest clothing — no adult body shapes, no bare midriffs, no revealing outfits. She has a blissful gentle expression, long flowing dark hair, a jeweled crown, and a radiant golden complexion. She has four arms — two hands showering golden coins, one holding a lotus flower, and one in a blessing gesture. She wears a full-length rich red-and-gold saree with an ornate border, a jeweled chest piece, wrist bangles, gold anklets, and sandals. She stands on a large pink lotus. Decorated with lotus motifs, gold coins, and a warm glowing halo. Place the figure on a classic round action-figure display pedestal with a smooth flat top and a slightly wider circular base — clean and simple in design. Set the entire scene against a solid plain background color (e.g. white, light grey, or a single bold color) with no gradients, patterns, or environment details. Fully optimized for 3D printing. Character should be barefoot with no footwear (no shoes, slippers, or sandals).</t>
         </is>
       </c>
     </row>

</xml_diff>